<commit_message>
Update CV and template
</commit_message>
<xml_diff>
--- a/input_blank/20230412_Onboarding_Template_Default_V3_forBackendUse.xlsx
+++ b/input_blank/20230412_Onboarding_Template_Default_V3_forBackendUse.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26903"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SangitaKumari\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raktimmaiti_mbp/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B4D25BA-D2EF-4497-8C5C-47FC641A760A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1083" documentId="13_ncr:1_{C2AE11D3-88BA-FA46-9561-7924B7B509F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D0E18EB-FA02-4EF6-8128-ECCBEF95DA44}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4660" yWindow="3020" windowWidth="28800" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Study_Experiment" sheetId="4" r:id="rId1"/>
@@ -18,6 +18,9 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -42,13 +45,13 @@
     <t>Study Type</t>
   </si>
   <si>
-    <t>ELN</t>
+    <t>UnileverStudyName</t>
   </si>
   <si>
     <t>Experiment Name</t>
   </si>
   <si>
-    <t>Experiment Technology</t>
+    <t>Assay Technology Type</t>
   </si>
   <si>
     <t>Experiment Type</t>
@@ -57,7 +60,7 @@
     <t>Platform</t>
   </si>
   <si>
-    <t>InvestigationType</t>
+    <t>PairedOrSingle</t>
   </si>
   <si>
     <t>Processing Status</t>
@@ -76,7 +79,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,8 +95,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -112,8 +124,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -136,20 +154,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -455,22 +489,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A48EB5A-D45B-4D2E-AF0D-50C88A468635}">
-  <dimension ref="A1:J31"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5703125" customWidth="1"/>
+    <col min="10" max="10" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15">
+    <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -495,10 +529,10 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -514,422 +548,35 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:10">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:10">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-    </row>
-    <row r="18" spans="1:10">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-    </row>
-    <row r="19" spans="1:10">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-    </row>
-    <row r="20" spans="1:10">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-    </row>
-    <row r="21" spans="1:10">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-    </row>
-    <row r="22" spans="1:10">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-    </row>
-    <row r="23" spans="1:10">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-    </row>
-    <row r="24" spans="1:10">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-    </row>
-    <row r="25" spans="1:10">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-    </row>
-    <row r="26" spans="1:10">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-    </row>
-    <row r="27" spans="1:10">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-    </row>
-    <row r="28" spans="1:10">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-    </row>
-    <row r="29" spans="1:10">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-    </row>
-    <row r="30" spans="1:10">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-    </row>
-    <row r="31" spans="1:10">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-    </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0"/>
+  <dataValidations count="3">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C30 D1:D1048576" xr:uid="{F3328EF8-467A-44B1-BB8F-A1E2DDED49B1}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B30 E2:H30" xr:uid="{D7AE5223-23A3-BC48-A670-292D3FE04DF7}">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J30" xr:uid="{4DAE9B66-8EA4-45B1-BB33-EDA7C873C20E}">
+      <formula1>_xlfn.ANCHORARRAY(#REF!)</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D7AE5223-23A3-BC48-A670-292D3FE04DF7}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>J2:J31</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{30DE47DC-7972-9949-9E50-63ACA098A773}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>H2:H31</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D44E2DBB-5C7D-C44D-9D44-6C10785348FD}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2:E31</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B4888CDB-5CAC-464E-A75B-545629014599}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2:F31</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FC84E200-C8E6-4340-8E31-E071990D54EC}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>G2:G31</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2A1686B7-09EC-9943-AB2F-3F1F9BEB4CA1}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>I2:I31</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C67B744-75A8-1E48-B34E-C50379535B08}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>B2:B31</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24544A25-124A-48F5-9C41-F8DFB0C5B9C1}">
   <dimension ref="A1:B5001"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
     </row>
@@ -20935,22 +20582,16 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0"/>
+  <dataValidations count="1">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1:XFD1" xr:uid="{B636C8CE-57F5-42FD-A63F-AA547C3EDD2D}"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A0F9FAEAB450C743A82F3E6ACA9501E3" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5bda77558553730cc6adee307ca99dcd">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f909b916-6d8f-4c4e-8026-d2dd022cb391" xmlns:ns3="e013bdf2-75c4-4dba-9483-b99bbda37e96" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="23a647b05e0f9c340e71388b0a57245d" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A0F9FAEAB450C743A82F3E6ACA9501E3" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fba29bf2eb12b184b6cdc215ae4b9b59">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f909b916-6d8f-4c4e-8026-d2dd022cb391" xmlns:ns3="e013bdf2-75c4-4dba-9483-b99bbda37e96" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="20590f377a1b291034f235da84ec3428" ns2:_="" ns3:_="">
     <xsd:import namespace="f909b916-6d8f-4c4e-8026-d2dd022cb391"/>
     <xsd:import namespace="e013bdf2-75c4-4dba-9483-b99bbda37e96"/>
     <xsd:element name="properties">
@@ -20974,6 +20615,7 @@
                 <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -21048,6 +20690,11 @@
     <xsd:element name="MediaLengthInSeconds" ma:index="23" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -21191,25 +20838,41 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="e013bdf2-75c4-4dba-9483-b99bbda37e96" xsi:nil="true"/>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="f909b916-6d8f-4c4e-8026-d2dd022cb391">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="e013bdf2-75c4-4dba-9483-b99bbda37e96">
+      <UserInfo>
+        <DisplayName>Denys Popko</DisplayName>
+        <AccountId>95</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
   </documentManagement>
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55F1472A-CF31-44CC-94B3-9E58178DD0AB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{935C932D-A4A1-4E50-A4CF-9A358E7DE507}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DDB049E-D376-42EA-81D6-FD4262EC4600}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BBF146-4DB2-45FB-A088-67BDF32BF239}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC383FB4-BB15-4E93-8531-3EA46DC7203F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55F1472A-CF31-44CC-94B3-9E58178DD0AB}"/>
 </file>
</xml_diff>